<commit_message>
feat(emotion): split neutral from calm (ADR-0021)
The former `calme` class held practical, neutral messages. It becomes
`neutre`, the low-confidence fallback, with a tiny grey animation; a new
`calme` class (peace, rest) gets 100 Claude-written examples (gate L29).
Legacy 8-label heads still read `calme` as neutral.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gdam7XiRLSp3sLTmHoRKeX
</commit_message>
<xml_diff>
--- a/data/emotions/dataset_emotions.xlsx
+++ b/data/emotions/dataset_emotions.xlsx
@@ -14,7 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="suspense" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tristesse" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="amour" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="calme" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="neutre" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="calme" sheetId="10" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tous_les_messages" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
@@ -1832,6 +1833,1237 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="0076D7C4"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B101"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="85" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>je suis posé dans mon lit avec un thé, tranquille</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>dimanche matin, pas de réveil, je profite</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>je regarde la pluie tomber par la fenêtre, ça m'apaise</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>je me sens zen aujourd'hui, rien ne me stresse</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>on est allongés dans l'herbe au parc, on regarde les nuages</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>j'ai enfin fini mes devoirs, je souffle un peu</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>balade au bord de l'eau, le bruit des vagues c'est trop apaisant</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>je lis mon livre sous la couette, je bouge plus</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>soirée tranquille à la maison, plaid et série</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>je viens de faire du yoga, je me sens léger</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>le soleil se couche sur la mer, c'est paisible</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>pas de pression ce week-end, je me repose</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>je respire un grand coup, tout va bien</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>on a marché en forêt, c'était calme et silencieux</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>ça fait du bien de rien faire de temps en temps</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>je suis sur le balcon avec de la musique douce</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>la maison est silencieuse, tout le monde dort, j'adore ce moment</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>je prends mon temps ce matin, petit déj au calme</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>t'inquiète on a le temps, on y va tranquillement</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>je suis détendu, la semaine est finie</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>bain chaud et bougies, je décompresse</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>on s'est posés au café, on a parlé doucement pendant des heures</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>je me sens apaisé depuis que j'ai parlé avec toi</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>le lac était lisse comme un miroir ce matin</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>journée cocooning, je sors pas de chez moi</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>je médite dix minutes avant de dormir, ça me calme</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>pas de stress, on verra demain</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>je suis dans le hamac au jardin, je pourrais y rester des heures</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>le chat dort sur mes genoux, je bouge pas</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>ce soir c'est tisane et dodo tôt</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>je me suis réveillé reposé pour une fois</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>on a pique-niqué tranquille au bord de la rivière</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>j'écoute le bruit de la pluie sur le toit, c'est trop reposant</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>rien de prévu aujourd'hui et ça me va très bien</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>je suis serein pour demain, je suis prêt</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>on fait une petite balade digestive, sans se presser</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>je regarde les étoiles depuis le jardin, tout est calme</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>vacances à la campagne, aucun bruit à part les oiseaux</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>j'ai éteint mon téléphone tout l'aprem, ça fait un bien fou</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>on prend le temps, rien ne presse</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>assis sur la plage, je regarde l'horizon</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>je dessine tranquillement dans ma chambre avec de la musique lo-fi</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>c'est doux comme soirée, j'aime bien</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>tout est rangé, la chambre est propre, je me sens apaisé</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>je suis posé au soleil, je recharge les batteries</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>on se fait une soirée chill sans écrans ?</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>je bois mon chocolat chaud en regardant la neige tomber</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>détends-toi, respire, ça va aller</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>le parc est vide ce matin, c'est hyper paisible</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>je me suis endormi sur le canapé, trop bien</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>on flâne en ville sans but précis</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>j'arrose les plantes, petit moment calme</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>la mer est calme aujourd'hui, on entend juste le vent</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>je suis bien installé, plus personne ne me dérange</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>je profite du silence avant que tout le monde se lève</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>on s'est allongés sur le sable chaud sans rien dire</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>j'ai pris un long bain, je suis tout relax</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>je me sens léger après cette marche</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>pas de cours demain, grasse mat tranquille</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>je suis en mode slow ce week-end</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>les feuilles tombent doucement, c'est apaisant à regarder</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>une soirée au coin du feu, rien de mieux</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>je lâche prise, je me prends plus la tête</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>on écoute un vieil album allongés par terre</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>petite sieste au soleil, le bonheur tranquille</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>tout est calme ici, ça repose</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>je respire l'air de la montagne, c'est pur et paisible</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>on joue aux cartes tranquillement en famille</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>je fais un puzzle en écoutant un podcast, zéro stress</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>j'ai pas envie de courir aujourd'hui, juste de me poser</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>la ville dort encore, je marche seul dans les rues vides</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>je suis apaisé, la dispute est réglée</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>on traîne en pyjama toute la journée</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>le bruit de la rivière me berce</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>on a regardé le coucher de soleil sans parler, c'était parfait</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>je prends une pause, je ferme les yeux deux minutes</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>je fais mes devoirs au calme à la bibliothèque</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>tranquille, je suis chez ma grand-mère à la campagne</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>on s'est fait un thé et on a papoté doucement</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>je suis dans ma bulle avec mes écouteurs, posé</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>je me sens en paix avec moi-même</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>ce matin j'ai bu mon café face au jardin, tout doux</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>on rentre à pied tranquillement, il fait bon</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>je profite de la fraîcheur du soir sur la terrasse</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>rien ne presse, prends ton temps</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>journée lente, je savoure</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>je suis au chaud sous mon plaid, il pleut dehors</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>on contemple la vue depuis le sommet, c'est tellement paisible</t>
+        </is>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>j'ai rangé mon bureau, je me sens plus serein</t>
+        </is>
+      </c>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>j'écoute du piano en m'endormant</t>
+        </is>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>on se pose sur un banc et on regarde les gens passer</t>
+        </is>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>je suis relax, aucune inquiétude</t>
+        </is>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>petite promenade à vélo sur le chemin du canal, tranquille</t>
+        </is>
+      </c>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>j'ai fait une liste, tout est sous contrôle, je suis apaisé</t>
+        </is>
+      </c>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>ce soir je reste au calme, j'ai besoin de souffler</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>le silence de la neige le matin c'est magique et apaisant</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>on lit chacun notre livre dans le salon, c'est doux</t>
+        </is>
+      </c>
+      <c r="B98" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>je fais des respirations profondes, ça va mieux</t>
+        </is>
+      </c>
+      <c r="B99" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>je suis bien, posé, sans rien attendre</t>
+        </is>
+      </c>
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="3" t="inlineStr">
+        <is>
+          <t>on s'est baignés dans le lac au lever du jour, tout était calme</t>
+        </is>
+      </c>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -9252,7 +10484,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9264,7 +10496,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9276,7 +10508,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9288,7 +10520,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9300,7 +10532,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9312,7 +10544,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9324,7 +10556,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9336,7 +10568,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9348,7 +10580,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9360,7 +10592,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9372,7 +10604,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9384,7 +10616,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9396,7 +10628,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9408,7 +10640,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9420,7 +10652,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9432,7 +10664,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9444,7 +10676,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9456,7 +10688,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9468,7 +10700,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9480,7 +10712,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9492,7 +10724,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9504,7 +10736,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9516,7 +10748,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9528,7 +10760,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9540,7 +10772,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9552,7 +10784,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9564,7 +10796,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9576,7 +10808,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9588,7 +10820,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9600,7 +10832,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9612,7 +10844,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9624,7 +10856,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9636,7 +10868,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9648,7 +10880,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9660,7 +10892,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9672,7 +10904,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9684,7 +10916,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9696,7 +10928,7 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9708,7 +10940,7 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9720,7 +10952,7 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9732,7 +10964,7 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9744,7 +10976,7 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9756,7 +10988,7 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9768,7 +11000,7 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9780,7 +11012,7 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9792,7 +11024,7 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9804,7 +11036,7 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9816,7 +11048,7 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9828,7 +11060,7 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9840,7 +11072,7 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9852,7 +11084,7 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9864,7 +11096,7 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9876,7 +11108,7 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9888,7 +11120,7 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9900,7 +11132,7 @@
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9912,7 +11144,7 @@
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9924,7 +11156,7 @@
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9936,7 +11168,7 @@
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9948,7 +11180,7 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9960,7 +11192,7 @@
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9972,7 +11204,7 @@
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9984,7 +11216,7 @@
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -9996,7 +11228,7 @@
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10008,7 +11240,7 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10020,7 +11252,7 @@
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10032,7 +11264,7 @@
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10044,7 +11276,7 @@
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10056,7 +11288,7 @@
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10068,7 +11300,7 @@
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10080,7 +11312,7 @@
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10092,7 +11324,7 @@
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10104,7 +11336,7 @@
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10116,7 +11348,7 @@
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10128,7 +11360,7 @@
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10140,7 +11372,7 @@
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10152,7 +11384,7 @@
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10164,7 +11396,7 @@
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10176,7 +11408,7 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10188,7 +11420,7 @@
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10200,7 +11432,7 @@
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10212,7 +11444,7 @@
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10224,7 +11456,7 @@
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10236,7 +11468,7 @@
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10248,7 +11480,7 @@
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10260,7 +11492,7 @@
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10272,7 +11504,7 @@
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10284,7 +11516,7 @@
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10296,7 +11528,7 @@
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10308,7 +11540,7 @@
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10320,7 +11552,7 @@
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10332,7 +11564,7 @@
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10344,7 +11576,7 @@
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10356,7 +11588,7 @@
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10368,7 +11600,7 @@
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10380,7 +11612,7 @@
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10392,7 +11624,7 @@
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10404,7 +11636,7 @@
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10416,7 +11648,7 @@
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10428,7 +11660,7 @@
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10440,7 +11672,7 @@
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -10456,7 +11688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B801"/>
+  <dimension ref="A1:B901"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="85" customWidth="1" min="1" max="1"/>
@@ -18883,7 +20115,7 @@
       </c>
       <c r="B702" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -18895,7 +20127,7 @@
       </c>
       <c r="B703" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -18907,7 +20139,7 @@
       </c>
       <c r="B704" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -18919,7 +20151,7 @@
       </c>
       <c r="B705" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -18931,7 +20163,7 @@
       </c>
       <c r="B706" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -18943,7 +20175,7 @@
       </c>
       <c r="B707" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -18955,7 +20187,7 @@
       </c>
       <c r="B708" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -18967,7 +20199,7 @@
       </c>
       <c r="B709" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -18979,7 +20211,7 @@
       </c>
       <c r="B710" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -18991,7 +20223,7 @@
       </c>
       <c r="B711" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19003,7 +20235,7 @@
       </c>
       <c r="B712" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19015,7 +20247,7 @@
       </c>
       <c r="B713" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19027,7 +20259,7 @@
       </c>
       <c r="B714" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19039,7 +20271,7 @@
       </c>
       <c r="B715" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19051,7 +20283,7 @@
       </c>
       <c r="B716" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19063,7 +20295,7 @@
       </c>
       <c r="B717" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19075,7 +20307,7 @@
       </c>
       <c r="B718" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19087,7 +20319,7 @@
       </c>
       <c r="B719" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19099,7 +20331,7 @@
       </c>
       <c r="B720" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19111,7 +20343,7 @@
       </c>
       <c r="B721" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19123,7 +20355,7 @@
       </c>
       <c r="B722" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19135,7 +20367,7 @@
       </c>
       <c r="B723" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19147,7 +20379,7 @@
       </c>
       <c r="B724" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19159,7 +20391,7 @@
       </c>
       <c r="B725" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19171,7 +20403,7 @@
       </c>
       <c r="B726" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19183,7 +20415,7 @@
       </c>
       <c r="B727" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19195,7 +20427,7 @@
       </c>
       <c r="B728" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19207,7 +20439,7 @@
       </c>
       <c r="B729" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19219,7 +20451,7 @@
       </c>
       <c r="B730" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19231,7 +20463,7 @@
       </c>
       <c r="B731" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19243,7 +20475,7 @@
       </c>
       <c r="B732" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19255,7 +20487,7 @@
       </c>
       <c r="B733" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19267,7 +20499,7 @@
       </c>
       <c r="B734" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19279,7 +20511,7 @@
       </c>
       <c r="B735" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19291,7 +20523,7 @@
       </c>
       <c r="B736" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19303,7 +20535,7 @@
       </c>
       <c r="B737" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19315,7 +20547,7 @@
       </c>
       <c r="B738" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19327,7 +20559,7 @@
       </c>
       <c r="B739" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19339,7 +20571,7 @@
       </c>
       <c r="B740" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19351,7 +20583,7 @@
       </c>
       <c r="B741" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19363,7 +20595,7 @@
       </c>
       <c r="B742" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19375,7 +20607,7 @@
       </c>
       <c r="B743" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19387,7 +20619,7 @@
       </c>
       <c r="B744" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19399,7 +20631,7 @@
       </c>
       <c r="B745" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19411,7 +20643,7 @@
       </c>
       <c r="B746" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19423,7 +20655,7 @@
       </c>
       <c r="B747" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19435,7 +20667,7 @@
       </c>
       <c r="B748" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19447,7 +20679,7 @@
       </c>
       <c r="B749" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19459,7 +20691,7 @@
       </c>
       <c r="B750" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19471,7 +20703,7 @@
       </c>
       <c r="B751" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19483,7 +20715,7 @@
       </c>
       <c r="B752" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19495,7 +20727,7 @@
       </c>
       <c r="B753" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19507,7 +20739,7 @@
       </c>
       <c r="B754" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19519,7 +20751,7 @@
       </c>
       <c r="B755" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19531,7 +20763,7 @@
       </c>
       <c r="B756" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19543,7 +20775,7 @@
       </c>
       <c r="B757" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19555,7 +20787,7 @@
       </c>
       <c r="B758" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19567,7 +20799,7 @@
       </c>
       <c r="B759" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19579,7 +20811,7 @@
       </c>
       <c r="B760" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19591,7 +20823,7 @@
       </c>
       <c r="B761" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19603,7 +20835,7 @@
       </c>
       <c r="B762" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19615,7 +20847,7 @@
       </c>
       <c r="B763" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19627,7 +20859,7 @@
       </c>
       <c r="B764" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19639,7 +20871,7 @@
       </c>
       <c r="B765" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19651,7 +20883,7 @@
       </c>
       <c r="B766" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19663,7 +20895,7 @@
       </c>
       <c r="B767" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19675,7 +20907,7 @@
       </c>
       <c r="B768" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19687,7 +20919,7 @@
       </c>
       <c r="B769" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19699,7 +20931,7 @@
       </c>
       <c r="B770" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19711,7 +20943,7 @@
       </c>
       <c r="B771" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19723,7 +20955,7 @@
       </c>
       <c r="B772" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19735,7 +20967,7 @@
       </c>
       <c r="B773" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19747,7 +20979,7 @@
       </c>
       <c r="B774" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19759,7 +20991,7 @@
       </c>
       <c r="B775" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19771,7 +21003,7 @@
       </c>
       <c r="B776" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19783,7 +21015,7 @@
       </c>
       <c r="B777" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19795,7 +21027,7 @@
       </c>
       <c r="B778" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19807,7 +21039,7 @@
       </c>
       <c r="B779" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19819,7 +21051,7 @@
       </c>
       <c r="B780" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19831,7 +21063,7 @@
       </c>
       <c r="B781" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19843,7 +21075,7 @@
       </c>
       <c r="B782" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19855,7 +21087,7 @@
       </c>
       <c r="B783" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19867,7 +21099,7 @@
       </c>
       <c r="B784" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19879,7 +21111,7 @@
       </c>
       <c r="B785" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19891,7 +21123,7 @@
       </c>
       <c r="B786" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19903,7 +21135,7 @@
       </c>
       <c r="B787" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19915,7 +21147,7 @@
       </c>
       <c r="B788" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19927,7 +21159,7 @@
       </c>
       <c r="B789" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19939,7 +21171,7 @@
       </c>
       <c r="B790" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19951,7 +21183,7 @@
       </c>
       <c r="B791" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19963,7 +21195,7 @@
       </c>
       <c r="B792" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19975,7 +21207,7 @@
       </c>
       <c r="B793" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19987,7 +21219,7 @@
       </c>
       <c r="B794" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -19999,7 +21231,7 @@
       </c>
       <c r="B795" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -20011,7 +21243,7 @@
       </c>
       <c r="B796" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -20023,7 +21255,7 @@
       </c>
       <c r="B797" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -20035,7 +21267,7 @@
       </c>
       <c r="B798" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -20047,7 +21279,7 @@
       </c>
       <c r="B799" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -20059,7 +21291,7 @@
       </c>
       <c r="B800" s="4" t="inlineStr">
         <is>
-          <t>calme</t>
+          <t>neutre</t>
         </is>
       </c>
     </row>
@@ -20070,6 +21302,1206 @@
         </is>
       </c>
       <c r="B801" s="4" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" s="3" t="inlineStr">
+        <is>
+          <t>je suis posé dans mon lit avec un thé, tranquille</t>
+        </is>
+      </c>
+      <c r="B802" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" s="3" t="inlineStr">
+        <is>
+          <t>dimanche matin, pas de réveil, je profite</t>
+        </is>
+      </c>
+      <c r="B803" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" s="3" t="inlineStr">
+        <is>
+          <t>je regarde la pluie tomber par la fenêtre, ça m'apaise</t>
+        </is>
+      </c>
+      <c r="B804" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" s="3" t="inlineStr">
+        <is>
+          <t>je me sens zen aujourd'hui, rien ne me stresse</t>
+        </is>
+      </c>
+      <c r="B805" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" s="3" t="inlineStr">
+        <is>
+          <t>on est allongés dans l'herbe au parc, on regarde les nuages</t>
+        </is>
+      </c>
+      <c r="B806" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" s="3" t="inlineStr">
+        <is>
+          <t>j'ai enfin fini mes devoirs, je souffle un peu</t>
+        </is>
+      </c>
+      <c r="B807" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" s="3" t="inlineStr">
+        <is>
+          <t>balade au bord de l'eau, le bruit des vagues c'est trop apaisant</t>
+        </is>
+      </c>
+      <c r="B808" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" s="3" t="inlineStr">
+        <is>
+          <t>je lis mon livre sous la couette, je bouge plus</t>
+        </is>
+      </c>
+      <c r="B809" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" s="3" t="inlineStr">
+        <is>
+          <t>soirée tranquille à la maison, plaid et série</t>
+        </is>
+      </c>
+      <c r="B810" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" s="3" t="inlineStr">
+        <is>
+          <t>je viens de faire du yoga, je me sens léger</t>
+        </is>
+      </c>
+      <c r="B811" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" s="3" t="inlineStr">
+        <is>
+          <t>le soleil se couche sur la mer, c'est paisible</t>
+        </is>
+      </c>
+      <c r="B812" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" s="3" t="inlineStr">
+        <is>
+          <t>pas de pression ce week-end, je me repose</t>
+        </is>
+      </c>
+      <c r="B813" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" s="3" t="inlineStr">
+        <is>
+          <t>je respire un grand coup, tout va bien</t>
+        </is>
+      </c>
+      <c r="B814" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" s="3" t="inlineStr">
+        <is>
+          <t>on a marché en forêt, c'était calme et silencieux</t>
+        </is>
+      </c>
+      <c r="B815" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" s="3" t="inlineStr">
+        <is>
+          <t>ça fait du bien de rien faire de temps en temps</t>
+        </is>
+      </c>
+      <c r="B816" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" s="3" t="inlineStr">
+        <is>
+          <t>je suis sur le balcon avec de la musique douce</t>
+        </is>
+      </c>
+      <c r="B817" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" s="3" t="inlineStr">
+        <is>
+          <t>la maison est silencieuse, tout le monde dort, j'adore ce moment</t>
+        </is>
+      </c>
+      <c r="B818" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" s="3" t="inlineStr">
+        <is>
+          <t>je prends mon temps ce matin, petit déj au calme</t>
+        </is>
+      </c>
+      <c r="B819" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" s="3" t="inlineStr">
+        <is>
+          <t>t'inquiète on a le temps, on y va tranquillement</t>
+        </is>
+      </c>
+      <c r="B820" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" s="3" t="inlineStr">
+        <is>
+          <t>je suis détendu, la semaine est finie</t>
+        </is>
+      </c>
+      <c r="B821" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" s="3" t="inlineStr">
+        <is>
+          <t>bain chaud et bougies, je décompresse</t>
+        </is>
+      </c>
+      <c r="B822" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" s="3" t="inlineStr">
+        <is>
+          <t>on s'est posés au café, on a parlé doucement pendant des heures</t>
+        </is>
+      </c>
+      <c r="B823" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" s="3" t="inlineStr">
+        <is>
+          <t>je me sens apaisé depuis que j'ai parlé avec toi</t>
+        </is>
+      </c>
+      <c r="B824" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" s="3" t="inlineStr">
+        <is>
+          <t>le lac était lisse comme un miroir ce matin</t>
+        </is>
+      </c>
+      <c r="B825" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" s="3" t="inlineStr">
+        <is>
+          <t>journée cocooning, je sors pas de chez moi</t>
+        </is>
+      </c>
+      <c r="B826" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" s="3" t="inlineStr">
+        <is>
+          <t>je médite dix minutes avant de dormir, ça me calme</t>
+        </is>
+      </c>
+      <c r="B827" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" s="3" t="inlineStr">
+        <is>
+          <t>pas de stress, on verra demain</t>
+        </is>
+      </c>
+      <c r="B828" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="3" t="inlineStr">
+        <is>
+          <t>je suis dans le hamac au jardin, je pourrais y rester des heures</t>
+        </is>
+      </c>
+      <c r="B829" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="3" t="inlineStr">
+        <is>
+          <t>le chat dort sur mes genoux, je bouge pas</t>
+        </is>
+      </c>
+      <c r="B830" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" s="3" t="inlineStr">
+        <is>
+          <t>ce soir c'est tisane et dodo tôt</t>
+        </is>
+      </c>
+      <c r="B831" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" s="3" t="inlineStr">
+        <is>
+          <t>je me suis réveillé reposé pour une fois</t>
+        </is>
+      </c>
+      <c r="B832" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" s="3" t="inlineStr">
+        <is>
+          <t>on a pique-niqué tranquille au bord de la rivière</t>
+        </is>
+      </c>
+      <c r="B833" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" s="3" t="inlineStr">
+        <is>
+          <t>j'écoute le bruit de la pluie sur le toit, c'est trop reposant</t>
+        </is>
+      </c>
+      <c r="B834" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" s="3" t="inlineStr">
+        <is>
+          <t>rien de prévu aujourd'hui et ça me va très bien</t>
+        </is>
+      </c>
+      <c r="B835" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" s="3" t="inlineStr">
+        <is>
+          <t>je suis serein pour demain, je suis prêt</t>
+        </is>
+      </c>
+      <c r="B836" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" s="3" t="inlineStr">
+        <is>
+          <t>on fait une petite balade digestive, sans se presser</t>
+        </is>
+      </c>
+      <c r="B837" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" s="3" t="inlineStr">
+        <is>
+          <t>je regarde les étoiles depuis le jardin, tout est calme</t>
+        </is>
+      </c>
+      <c r="B838" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" s="3" t="inlineStr">
+        <is>
+          <t>vacances à la campagne, aucun bruit à part les oiseaux</t>
+        </is>
+      </c>
+      <c r="B839" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" s="3" t="inlineStr">
+        <is>
+          <t>j'ai éteint mon téléphone tout l'aprem, ça fait un bien fou</t>
+        </is>
+      </c>
+      <c r="B840" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" s="3" t="inlineStr">
+        <is>
+          <t>on prend le temps, rien ne presse</t>
+        </is>
+      </c>
+      <c r="B841" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" s="3" t="inlineStr">
+        <is>
+          <t>assis sur la plage, je regarde l'horizon</t>
+        </is>
+      </c>
+      <c r="B842" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" s="3" t="inlineStr">
+        <is>
+          <t>je dessine tranquillement dans ma chambre avec de la musique lo-fi</t>
+        </is>
+      </c>
+      <c r="B843" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" s="3" t="inlineStr">
+        <is>
+          <t>c'est doux comme soirée, j'aime bien</t>
+        </is>
+      </c>
+      <c r="B844" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" s="3" t="inlineStr">
+        <is>
+          <t>tout est rangé, la chambre est propre, je me sens apaisé</t>
+        </is>
+      </c>
+      <c r="B845" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" s="3" t="inlineStr">
+        <is>
+          <t>je suis posé au soleil, je recharge les batteries</t>
+        </is>
+      </c>
+      <c r="B846" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" s="3" t="inlineStr">
+        <is>
+          <t>on se fait une soirée chill sans écrans ?</t>
+        </is>
+      </c>
+      <c r="B847" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" s="3" t="inlineStr">
+        <is>
+          <t>je bois mon chocolat chaud en regardant la neige tomber</t>
+        </is>
+      </c>
+      <c r="B848" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" s="3" t="inlineStr">
+        <is>
+          <t>détends-toi, respire, ça va aller</t>
+        </is>
+      </c>
+      <c r="B849" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" s="3" t="inlineStr">
+        <is>
+          <t>le parc est vide ce matin, c'est hyper paisible</t>
+        </is>
+      </c>
+      <c r="B850" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" s="3" t="inlineStr">
+        <is>
+          <t>je me suis endormi sur le canapé, trop bien</t>
+        </is>
+      </c>
+      <c r="B851" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" s="3" t="inlineStr">
+        <is>
+          <t>on flâne en ville sans but précis</t>
+        </is>
+      </c>
+      <c r="B852" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" s="3" t="inlineStr">
+        <is>
+          <t>j'arrose les plantes, petit moment calme</t>
+        </is>
+      </c>
+      <c r="B853" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" s="3" t="inlineStr">
+        <is>
+          <t>la mer est calme aujourd'hui, on entend juste le vent</t>
+        </is>
+      </c>
+      <c r="B854" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" s="3" t="inlineStr">
+        <is>
+          <t>je suis bien installé, plus personne ne me dérange</t>
+        </is>
+      </c>
+      <c r="B855" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" s="3" t="inlineStr">
+        <is>
+          <t>je profite du silence avant que tout le monde se lève</t>
+        </is>
+      </c>
+      <c r="B856" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" s="3" t="inlineStr">
+        <is>
+          <t>on s'est allongés sur le sable chaud sans rien dire</t>
+        </is>
+      </c>
+      <c r="B857" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" s="3" t="inlineStr">
+        <is>
+          <t>j'ai pris un long bain, je suis tout relax</t>
+        </is>
+      </c>
+      <c r="B858" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" s="3" t="inlineStr">
+        <is>
+          <t>je me sens léger après cette marche</t>
+        </is>
+      </c>
+      <c r="B859" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" s="3" t="inlineStr">
+        <is>
+          <t>pas de cours demain, grasse mat tranquille</t>
+        </is>
+      </c>
+      <c r="B860" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" s="3" t="inlineStr">
+        <is>
+          <t>je suis en mode slow ce week-end</t>
+        </is>
+      </c>
+      <c r="B861" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" s="3" t="inlineStr">
+        <is>
+          <t>les feuilles tombent doucement, c'est apaisant à regarder</t>
+        </is>
+      </c>
+      <c r="B862" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" s="3" t="inlineStr">
+        <is>
+          <t>une soirée au coin du feu, rien de mieux</t>
+        </is>
+      </c>
+      <c r="B863" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" s="3" t="inlineStr">
+        <is>
+          <t>je lâche prise, je me prends plus la tête</t>
+        </is>
+      </c>
+      <c r="B864" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" s="3" t="inlineStr">
+        <is>
+          <t>on écoute un vieil album allongés par terre</t>
+        </is>
+      </c>
+      <c r="B865" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" s="3" t="inlineStr">
+        <is>
+          <t>petite sieste au soleil, le bonheur tranquille</t>
+        </is>
+      </c>
+      <c r="B866" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" s="3" t="inlineStr">
+        <is>
+          <t>tout est calme ici, ça repose</t>
+        </is>
+      </c>
+      <c r="B867" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" s="3" t="inlineStr">
+        <is>
+          <t>je respire l'air de la montagne, c'est pur et paisible</t>
+        </is>
+      </c>
+      <c r="B868" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" s="3" t="inlineStr">
+        <is>
+          <t>on joue aux cartes tranquillement en famille</t>
+        </is>
+      </c>
+      <c r="B869" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" s="3" t="inlineStr">
+        <is>
+          <t>je fais un puzzle en écoutant un podcast, zéro stress</t>
+        </is>
+      </c>
+      <c r="B870" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" s="3" t="inlineStr">
+        <is>
+          <t>j'ai pas envie de courir aujourd'hui, juste de me poser</t>
+        </is>
+      </c>
+      <c r="B871" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" s="3" t="inlineStr">
+        <is>
+          <t>la ville dort encore, je marche seul dans les rues vides</t>
+        </is>
+      </c>
+      <c r="B872" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" s="3" t="inlineStr">
+        <is>
+          <t>je suis apaisé, la dispute est réglée</t>
+        </is>
+      </c>
+      <c r="B873" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" s="3" t="inlineStr">
+        <is>
+          <t>on traîne en pyjama toute la journée</t>
+        </is>
+      </c>
+      <c r="B874" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" s="3" t="inlineStr">
+        <is>
+          <t>le bruit de la rivière me berce</t>
+        </is>
+      </c>
+      <c r="B875" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" s="3" t="inlineStr">
+        <is>
+          <t>on a regardé le coucher de soleil sans parler, c'était parfait</t>
+        </is>
+      </c>
+      <c r="B876" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" s="3" t="inlineStr">
+        <is>
+          <t>je prends une pause, je ferme les yeux deux minutes</t>
+        </is>
+      </c>
+      <c r="B877" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" s="3" t="inlineStr">
+        <is>
+          <t>je fais mes devoirs au calme à la bibliothèque</t>
+        </is>
+      </c>
+      <c r="B878" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" s="3" t="inlineStr">
+        <is>
+          <t>tranquille, je suis chez ma grand-mère à la campagne</t>
+        </is>
+      </c>
+      <c r="B879" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" s="3" t="inlineStr">
+        <is>
+          <t>on s'est fait un thé et on a papoté doucement</t>
+        </is>
+      </c>
+      <c r="B880" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" s="3" t="inlineStr">
+        <is>
+          <t>je suis dans ma bulle avec mes écouteurs, posé</t>
+        </is>
+      </c>
+      <c r="B881" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" s="3" t="inlineStr">
+        <is>
+          <t>je me sens en paix avec moi-même</t>
+        </is>
+      </c>
+      <c r="B882" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" s="3" t="inlineStr">
+        <is>
+          <t>ce matin j'ai bu mon café face au jardin, tout doux</t>
+        </is>
+      </c>
+      <c r="B883" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" s="3" t="inlineStr">
+        <is>
+          <t>on rentre à pied tranquillement, il fait bon</t>
+        </is>
+      </c>
+      <c r="B884" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" s="3" t="inlineStr">
+        <is>
+          <t>je profite de la fraîcheur du soir sur la terrasse</t>
+        </is>
+      </c>
+      <c r="B885" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" s="3" t="inlineStr">
+        <is>
+          <t>rien ne presse, prends ton temps</t>
+        </is>
+      </c>
+      <c r="B886" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" s="3" t="inlineStr">
+        <is>
+          <t>journée lente, je savoure</t>
+        </is>
+      </c>
+      <c r="B887" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" s="3" t="inlineStr">
+        <is>
+          <t>je suis au chaud sous mon plaid, il pleut dehors</t>
+        </is>
+      </c>
+      <c r="B888" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" s="3" t="inlineStr">
+        <is>
+          <t>on contemple la vue depuis le sommet, c'est tellement paisible</t>
+        </is>
+      </c>
+      <c r="B889" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" s="3" t="inlineStr">
+        <is>
+          <t>j'ai rangé mon bureau, je me sens plus serein</t>
+        </is>
+      </c>
+      <c r="B890" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" s="3" t="inlineStr">
+        <is>
+          <t>j'écoute du piano en m'endormant</t>
+        </is>
+      </c>
+      <c r="B891" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" s="3" t="inlineStr">
+        <is>
+          <t>on se pose sur un banc et on regarde les gens passer</t>
+        </is>
+      </c>
+      <c r="B892" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" s="3" t="inlineStr">
+        <is>
+          <t>je suis relax, aucune inquiétude</t>
+        </is>
+      </c>
+      <c r="B893" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" s="3" t="inlineStr">
+        <is>
+          <t>petite promenade à vélo sur le chemin du canal, tranquille</t>
+        </is>
+      </c>
+      <c r="B894" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" s="3" t="inlineStr">
+        <is>
+          <t>j'ai fait une liste, tout est sous contrôle, je suis apaisé</t>
+        </is>
+      </c>
+      <c r="B895" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" s="3" t="inlineStr">
+        <is>
+          <t>ce soir je reste au calme, j'ai besoin de souffler</t>
+        </is>
+      </c>
+      <c r="B896" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" s="3" t="inlineStr">
+        <is>
+          <t>le silence de la neige le matin c'est magique et apaisant</t>
+        </is>
+      </c>
+      <c r="B897" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" s="3" t="inlineStr">
+        <is>
+          <t>on lit chacun notre livre dans le salon, c'est doux</t>
+        </is>
+      </c>
+      <c r="B898" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" s="3" t="inlineStr">
+        <is>
+          <t>je fais des respirations profondes, ça va mieux</t>
+        </is>
+      </c>
+      <c r="B899" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" s="3" t="inlineStr">
+        <is>
+          <t>je suis bien, posé, sans rien attendre</t>
+        </is>
+      </c>
+      <c r="B900" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" s="3" t="inlineStr">
+        <is>
+          <t>on s'est baignés dans le lac au lever du jour, tout était calme</t>
+        </is>
+      </c>
+      <c r="B901" s="4" t="inlineStr">
         <is>
           <t>calme</t>
         </is>

</xml_diff>

<commit_message>
feat(data): add emoji examples to every emotion sheet
90 short messages with emoji, 10 per category, written by Claude at the
owner's request (L29). On a separate hand-written emoji probe, 👍 and 👌
now read as neutre and 🙈 as genance; dev_v1 accuracy 84.3% -> 85.7%.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gdam7XiRLSp3sLTmHoRKeX
</commit_message>
<xml_diff>
--- a/data/emotions/dataset_emotions.xlsx
+++ b/data/emotions/dataset_emotions.xlsx
@@ -609,7 +609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B101"/>
+  <dimension ref="A1:B111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="85" customWidth="1" min="1" max="1"/>
@@ -1823,6 +1823,126 @@
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>joie</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>J'ai eu mon permis 😂🎉</t>
+        </is>
+      </c>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>joie</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>trop content de te revoir demain 😁</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>joie</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>on a gagné le match 🥳</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>joie</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>mdr ta blague m'a tuée 🤣</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>joie</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>c'est les vacances enfin 😄☀️</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>joie</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>j'ai réussi mon contrôle de maths 😊</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>joie</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>ma sœur a eu son bac 🎉🎉</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>joie</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>hâte de fêter ça avec vous 🥳</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>joie</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>ce film était trop drôle 😂</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>joie</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>j'ai trouvé le cadeau parfait 😁</t>
+        </is>
+      </c>
+      <c r="B111" s="4" t="inlineStr">
         <is>
           <t>joie</t>
         </is>
@@ -1840,7 +1960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B101"/>
+  <dimension ref="A1:B111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="85" customWidth="1" min="1" max="1"/>
@@ -3054,6 +3174,126 @@
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>petite balade au bord du lac 🌿</t>
+        </is>
+      </c>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>je me pose avec un thé 🍵</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>soirée tranquille sous la couette 😌</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>je respire enfin 😌</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>je vais faire une sieste 😴</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>le coucher de soleil est magnifique 🌅</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>dimanche cocooning 🛋️</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>lecture au calme ce soir 📖</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>rien de prévu, juste me reposer 😴</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>méditation du matin 🧘</t>
+        </is>
+      </c>
+      <c r="B111" s="4" t="inlineStr">
         <is>
           <t>calme</t>
         </is>
@@ -3071,7 +3311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B101"/>
+  <dimension ref="A1:B111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="85" customWidth="1" min="1" max="1"/>
@@ -4285,6 +4525,126 @@
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>genance</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>j'ai appelé la prof maman 🙈</t>
+        </is>
+      </c>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>genance</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>je suis tombé devant tout le monde 😳</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>genance</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>oups mauvaise conversation 😅</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>genance</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>j'ai envoyé le message au mauvais groupe 🙈</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>genance</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>je savais plus où me mettre 😳</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>genance</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>mon père a dansé devant mes potes 🫣</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>genance</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>j'ai fait coucou à quelqu'un qui saluait pas moi 😅</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>genance</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>je suis devenu tout rouge 😳</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>genance</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>trop la honte j'ai bégayé à l'oral 🙈</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>genance</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>mon ventre a gargouillé en plein silence 🫣</t>
+        </is>
+      </c>
+      <c r="B111" s="4" t="inlineStr">
         <is>
           <t>genance</t>
         </is>
@@ -4302,7 +4662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B101"/>
+  <dimension ref="A1:B111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="85" customWidth="1" min="1" max="1"/>
@@ -5516,6 +5876,126 @@
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>colere</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>tu m'as encore posé un lapin 😡</t>
+        </is>
+      </c>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>colere</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>j'en ai marre de tes mensonges 🤬</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>colere</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>arrête de me prendre pour une idiote 😠</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>colere</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>il a cassé mon téléphone 😤</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>colere</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>personne m'écoute ici 😡</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>colere</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>t'avais promis et t'as rien fait 😠</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>colere</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>ils ont encore annulé sans prévenir 🤬</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>colere</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>me parle plus jamais comme ça 😤</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>colere</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>j'ai attendu une heure pour rien 😡</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>colere</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>c'est injuste j'ai rien fait 😠</t>
+        </is>
+      </c>
+      <c r="B111" s="4" t="inlineStr">
         <is>
           <t>colere</t>
         </is>
@@ -5533,7 +6013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B101"/>
+  <dimension ref="A1:B111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="85" customWidth="1" min="1" max="1"/>
@@ -6747,6 +7227,126 @@
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>energie</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>allez on se donne à fond 💪🔥</t>
+        </is>
+      </c>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>energie</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>go go go on va tout casser 🔥</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>energie</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>prêt pour la soirée de folie ⚡</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>energie</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>on lâche rien les gars 💪</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>energie</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>entraînement de malade aujourd'hui 🔥</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>energie</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>let's go le match commence 🚀</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>energie</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>je suis chaud pour ce soir ⚡🔥</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>energie</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>on y va à fond 🚀</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>energie</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>full motivation ce matin 💪</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>energie</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>ce concert va être énorme 🔥🤘</t>
+        </is>
+      </c>
+      <c r="B111" s="4" t="inlineStr">
         <is>
           <t>energie</t>
         </is>
@@ -6764,7 +7364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B101"/>
+  <dimension ref="A1:B111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="85" customWidth="1" min="1" max="1"/>
@@ -7978,6 +8578,126 @@
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>suspense</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>devine ce qui vient de se passer 👀</t>
+        </is>
+      </c>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>suspense</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>j'ai un secret à te dire 🤫</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>suspense</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>attends tu vas jamais croire ça 😱</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>suspense</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>les résultats tombent dans une heure 😬</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>suspense</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>qui a envoyé ce message ?? 👀</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>suspense</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>il se passe un truc bizarre dehors 😨</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>suspense</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>j'ose pas ouvrir la lettre 😬</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>suspense</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>tu sais pas qui j'ai croisé 👀</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>suspense</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>la fin de l'épisode 😱 vite la suite</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>suspense</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>j'attends sa réponse 😰</t>
+        </is>
+      </c>
+      <c r="B111" s="4" t="inlineStr">
         <is>
           <t>suspense</t>
         </is>
@@ -7995,7 +8715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B101"/>
+  <dimension ref="A1:B111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="85" customWidth="1" min="1" max="1"/>
@@ -9209,6 +9929,126 @@
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>tristesse</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>mon chat est mort ce matin 😢</t>
+        </is>
+      </c>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>tristesse</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>elle m'a quitté 💔</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>tristesse</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>je me sens trop seul ce soir 😞</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>tristesse</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>j'ai raté mon examen 😭</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>tristesse</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>tu vas me manquer 😢</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>tristesse</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>personne est venu à mon anniv 😔</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>tristesse</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>mon meilleur ami déménage 😭</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>tristesse</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>j'ai pas été pris dans l'équipe 😞</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>tristesse</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>journée horrible j'ai envie de pleurer 😢</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>tristesse</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>mes parents se séparent 💔</t>
+        </is>
+      </c>
+      <c r="B111" s="4" t="inlineStr">
         <is>
           <t>tristesse</t>
         </is>
@@ -9226,7 +10066,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B101"/>
+  <dimension ref="A1:B111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="85" customWidth="1" min="1" max="1"/>
@@ -10440,6 +11280,126 @@
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>amour</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>je pense à toi 💕</t>
+        </is>
+      </c>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>amour</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>t'es la personne la plus importante pour moi ❤️</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>amour</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>tu me manques mon cœur 😘</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>amour</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>je t'aime fort 💖</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>amour</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>merci d'être là pour moi 🥰</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>amour</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>bonne nuit mon amour 😘</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>amour</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>trop hâte de te serrer dans mes bras 💞</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>amour</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>t'es trop mignon 😍</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>amour</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>je suis fou de toi ❤️</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>amour</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>mon cœur est à toi 💘</t>
+        </is>
+      </c>
+      <c r="B111" s="4" t="inlineStr">
         <is>
           <t>amour</t>
         </is>
@@ -10457,7 +11417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B101"/>
+  <dimension ref="A1:B111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="85" customWidth="1" min="1" max="1"/>
@@ -11671,6 +12631,126 @@
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>ok 👍</t>
+        </is>
+      </c>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>je suis arrivé 📍</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>rdv à 14h devant la gare 👍</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>c'est noté 👌</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>tu peux m'envoyer le lien ? 📎</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>je t'appelle après le cours 📞</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>le bus a 5 min de retard 🚌</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>j'ai pris le pain 🥖</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>réunion déplacée à jeudi 📅</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>d'accord pour demain 👌</t>
+        </is>
+      </c>
+      <c r="B111" s="4" t="inlineStr">
         <is>
           <t>neutre</t>
         </is>

</xml_diff>